<commit_message>
Added a script to read, process and export raw prevah discharge.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noahnydegger/GitHub/ETH/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0C83A9-2D5A-E64E-BAD5-491C9023EE95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E762FE9-D9E6-3640-B2E3-56DE54CAD11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24520" yWindow="22360" windowWidth="28060" windowHeight="17460" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="-30120" yWindow="15320" windowWidth="28060" windowHeight="17460" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
   <si>
     <t>Date</t>
   </si>
@@ -87,6 +87,18 @@
   </si>
   <si>
     <t>Hd_2050, Hn_2050, Md_2050, Mn_2050</t>
+  </si>
+  <si>
+    <t>Hd_2050</t>
+  </si>
+  <si>
+    <t>TGl200 ThS200 Rhb200 BEN200 BiS200 Bod400 EmW200 HiR200 LaP200 Lim200 NeS200</t>
+  </si>
+  <si>
+    <t>Testrun future scenario for Rheinblick Meeting</t>
+  </si>
+  <si>
+    <t>NoW200 KEm200 SeD200 SSG200 Thu200 VoA200 VoR200 WaS200</t>
   </si>
 </sst>
 </file>
@@ -94,10 +106,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-CH,1]hh:mm;@"/>
-    <numFmt numFmtId="170" formatCode="[$]dd/mm/yyyy;@" x16r2:formatCode16="[$-en-CH,1]dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-CH,1]hh:mm;@"/>
+    <numFmt numFmtId="165" formatCode="[$]dd/mm/yyyy;@" x16r2:formatCode16="[$-en-CH,1]dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -117,6 +129,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFCE9178"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -139,14 +157,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -481,13 +498,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.1640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="4"/>
     <col min="3" max="4" width="10.83203125" style="3"/>
-    <col min="5" max="6" width="10.83203125" style="6"/>
+    <col min="5" max="6" width="10.83203125" style="2"/>
     <col min="7" max="7" width="43.33203125" style="2" customWidth="1"/>
     <col min="8" max="16384" width="10.83203125" style="2"/>
   </cols>
@@ -505,10 +522,10 @@
       <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -534,10 +551,10 @@
       <c r="D2" s="3">
         <v>0.7583333333333333</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="2">
         <v>1921889</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="2">
         <v>1921917</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -563,10 +580,10 @@
       <c r="D3" s="3">
         <v>0.44583333333333336</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="2">
         <v>1922757</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="2">
         <v>1922917</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -592,10 +609,10 @@
       <c r="D4" s="3">
         <v>0.88402777777777775</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="2">
         <v>1923986</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="2">
         <v>1923993</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -621,10 +638,10 @@
       <c r="D5" s="3">
         <v>0.4909722222222222</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="2">
         <v>1928244</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="2">
         <v>1928279</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -636,6 +653,64 @@
       <c r="I5" s="2" t="s">
         <v>12</v>
       </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="4">
+        <v>45722</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.5854166666666667</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.64722222222222225</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1940153</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1940253</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4">
+        <v>45723</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.73541666666666672</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1940853</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I8" s="5"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="I9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
modified processing function to add a column that specifies warmup vs. simulation period and changes Bod200 to Bod400.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noahnydegger/GitHub/ETH/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E762FE9-D9E6-3640-B2E3-56DE54CAD11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398E17B7-C299-124F-9691-2089DD3DCDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30120" yWindow="15320" windowWidth="28060" windowHeight="17460" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="-35940" yWindow="3280" windowWidth="28060" windowHeight="17460" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
   <si>
     <t>Date</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t>NoW200 KEm200 SeD200 SSG200 Thu200 VoA200 VoR200 WaS200</t>
+  </si>
+  <si>
+    <t>Reference Run with corrected lapse rate</t>
+  </si>
+  <si>
+    <t>alle</t>
   </si>
 </sst>
 </file>
@@ -109,7 +115,7 @@
     <numFmt numFmtId="164" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-CH,1]hh:mm;@"/>
     <numFmt numFmtId="165" formatCode="[$]dd/mm/yyyy;@" x16r2:formatCode16="[$-en-CH,1]dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -129,12 +135,6 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFCE9178"/>
-      <name val="Menlo"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -157,13 +157,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.1640625" style="2" customWidth="1"/>
@@ -707,10 +706,33 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I8" s="5"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I9" s="5"/>
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4">
+        <v>45736</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.46388888888888891</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.57152777777777775</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1969570</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1969728</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
new functions to compare meteo raster and changed plot functions.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398E17B7-C299-124F-9691-2089DD3DCDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006E0981-267E-934C-A7F0-40BDA4C6E95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35940" yWindow="3280" windowWidth="28060" windowHeight="17460" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -105,6 +105,15 @@
   </si>
   <si>
     <t>alle</t>
+  </si>
+  <si>
+    <t>sund BC test</t>
+  </si>
+  <si>
+    <t>Hd_2100</t>
+  </si>
+  <si>
+    <t>ThS200 Thu200</t>
   </si>
 </sst>
 </file>
@@ -497,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="38.1640625" style="2" customWidth="1"/>
@@ -734,6 +743,35 @@
         <v>22</v>
       </c>
     </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="4">
+        <v>45743</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.35069444444444442</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1972159</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1972174</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
read ch2018 meteo and glacier data to a DT. find best matching gl chain. radg to sund conversion Rscripts from Massimiliano.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006E0981-267E-934C-A7F0-40BDA4C6E95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AEA89BA-409D-BC45-BD9E-FCC082354031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="6000" yWindow="1460" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -114,6 +114,15 @@
   </si>
   <si>
     <t>ThS200 Thu200</t>
+  </si>
+  <si>
+    <t>Andelfingen Hn2100 Opening Seminar</t>
+  </si>
+  <si>
+    <t>Hn_2100</t>
+  </si>
+  <si>
+    <t>Andelfingen Hn2100 Opening Seminar - did not work</t>
   </si>
 </sst>
 </file>
@@ -506,10 +515,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.1640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="4"/>
     <col min="3" max="4" width="10.83203125" style="3"/>
     <col min="5" max="6" width="10.83203125" style="2"/>
@@ -772,6 +781,58 @@
         <v>25</v>
       </c>
     </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="4">
+        <v>45754</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.46527777777777779</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1995851</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="4">
+        <v>45755</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0.44305555555555554</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.45555555555555555</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1996132</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1996148</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
snapshot before increasing disk image size.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AEA89BA-409D-BC45-BD9E-FCC082354031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A6FCDE0-8081-F048-AF2F-C4A844F6D7CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6000" yWindow="1460" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="30">
   <si>
     <t>Date</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>Andelfingen Hn2100 Opening Seminar - did not work</t>
+  </si>
+  <si>
+    <t>Glacier Comparison - no lapse rate</t>
   </si>
 </sst>
 </file>
@@ -515,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
@@ -644,7 +647,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B5" s="4">
         <v>45719</v>
@@ -831,6 +834,17 @@
       </c>
       <c r="I11" s="2" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed read_prevah_all_components to export scenario_horizon as individual .rds and .csv
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A6FCDE0-8081-F048-AF2F-C4A844F6D7CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED6A0C8-AE86-0E48-9085-E950A2E9AAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6000" yWindow="1460" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
   <si>
     <t>Date</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>Glacier Comparison - no lapse rate</t>
+  </si>
+  <si>
+    <t>Hd_2050, Hd_2150, Hn_2050, Hn_2150, L_2033, Ld_2100, Ln_2100, Md_2050, Md_2100, Md_2150, Mn_2050, Mn_2100, Mn_2150</t>
   </si>
 </sst>
 </file>
@@ -840,6 +843,18 @@
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="B12" s="4">
+        <v>45757</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.66388888888888886</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1997212</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="H12" s="2" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
sund bc done for a first iteration. also analyse effect on future.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED6A0C8-AE86-0E48-9085-E950A2E9AAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F11D40-9417-E74D-B7DB-D4F80FA39086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="1460" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="2380" yWindow="840" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Hd_2050, Hd_2150, Hn_2050, Hn_2150, L_2033, Ld_2100, Ln_2100, Md_2050, Md_2100, Md_2150, Mn_2050, Mn_2100, Mn_2150</t>
+  </si>
+  <si>
+    <t>Mn_2100, Mn_2150</t>
+  </si>
+  <si>
+    <t>Glacier Comparison, were not generated before</t>
   </si>
 </sst>
 </file>
@@ -521,14 +527,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="4"/>
     <col min="3" max="4" width="10.83203125" style="3"/>
     <col min="5" max="6" width="10.83203125" style="2"/>
-    <col min="7" max="7" width="43.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="106.33203125" style="2" customWidth="1"/>
     <col min="8" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
@@ -862,6 +868,23 @@
         <v>12</v>
       </c>
     </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="4">
+        <v>45764</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0.68333333333333335</v>
+      </c>
+      <c r="E13" s="2">
+        <v>2000048</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
selected glchains for knmi scenarios. per ensemble for 2033 to 2100 and per scenario for 2150 and reference. Script to check if all jobs did run until the last day.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F11D40-9417-E74D-B7DB-D4F80FA39086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5C7968-F8EF-7F40-92B0-7CDFF1D8604B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2380" yWindow="840" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -135,6 +135,42 @@
   </si>
   <si>
     <t>Glacier Comparison, were not generated before</t>
+  </si>
+  <si>
+    <t>Glacier Comparison, stopped at year 2043</t>
+  </si>
+  <si>
+    <t>Hn_2050</t>
+  </si>
+  <si>
+    <t>Glacier Comparison, stopped before finish</t>
+  </si>
+  <si>
+    <t>L_2033</t>
+  </si>
+  <si>
+    <t>5..8</t>
+  </si>
+  <si>
+    <t>Md_2100</t>
+  </si>
+  <si>
+    <t>Ld_2100</t>
+  </si>
+  <si>
+    <t>2..8</t>
+  </si>
+  <si>
+    <t>Ln_2100</t>
+  </si>
+  <si>
+    <t>2..4</t>
+  </si>
+  <si>
+    <t>Hd_2150</t>
+  </si>
+  <si>
+    <t>4..8</t>
   </si>
 </sst>
 </file>
@@ -187,12 +223,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
@@ -589,7 +626,7 @@
       <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -618,7 +655,7 @@
       <c r="G3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I3" s="2" t="s">
@@ -647,7 +684,7 @@
       <c r="G4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -676,7 +713,7 @@
       <c r="G5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -705,7 +742,7 @@
       <c r="G6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -728,7 +765,7 @@
       <c r="G7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I7" s="2" t="s">
@@ -757,7 +794,7 @@
       <c r="G8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -786,7 +823,7 @@
       <c r="G9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -809,7 +846,7 @@
       <c r="G10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I10" s="2" t="s">
@@ -838,7 +875,7 @@
       <c r="G11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I11" s="2" t="s">
@@ -861,7 +898,7 @@
       <c r="G12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I12" s="2" t="s">
@@ -883,6 +920,174 @@
       </c>
       <c r="G13" s="2" t="s">
         <v>31</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="4">
+        <v>45769</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0.64097222222222228</v>
+      </c>
+      <c r="E14" s="2">
+        <v>2001612</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="4">
+        <v>45771</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.37777777777777777</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.37986111111111109</v>
+      </c>
+      <c r="E15" s="2">
+        <v>2002868</v>
+      </c>
+      <c r="F15" s="2">
+        <v>2002873</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="4">
+        <v>45771</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="E16" s="2">
+        <v>2002881</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" s="5">
+        <v>2</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="4">
+        <v>45771</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.38750000000000001</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.39166666666666666</v>
+      </c>
+      <c r="E17" s="2">
+        <v>2002882</v>
+      </c>
+      <c r="F17" s="2">
+        <v>2002891</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="4">
+        <v>45771</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.39305555555555555</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.39444444444444443</v>
+      </c>
+      <c r="E18" s="2">
+        <v>2002892</v>
+      </c>
+      <c r="F18" s="2">
+        <v>2002895</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="4">
+        <v>45771</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.39861111111111114</v>
+      </c>
+      <c r="E19" s="2">
+        <v>2002897</v>
+      </c>
+      <c r="F19" s="2">
+        <v>2002903</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adjusted all plotting functions with a plot_dir. Generated sdbc.2km files. Changed the bash scripts to copy to and from hyperion. Added the column run_type to the read_raw_prevah functions.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5C7968-F8EF-7F40-92B0-7CDFF1D8604B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314436CA-9D01-464E-9EDF-277BD371C775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2380" yWindow="840" windowWidth="30240" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="102980" yWindow="21860" windowWidth="30240" windowHeight="17360" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
   <si>
     <t>Date</t>
   </si>
@@ -171,6 +171,18 @@
   </si>
   <si>
     <t>4..8</t>
+  </si>
+  <si>
+    <t>Glacier Comparison - test run</t>
+  </si>
+  <si>
+    <t>Hd_2050, Hd_2100, Hd_2150</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Rhb200</t>
   </si>
 </sst>
 </file>
@@ -223,13 +235,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -564,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
@@ -572,7 +585,8 @@
     <col min="3" max="4" width="10.83203125" style="3"/>
     <col min="5" max="6" width="10.83203125" style="2"/>
     <col min="7" max="7" width="106.33203125" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="2"/>
+    <col min="8" max="8" width="10.83203125" style="5"/>
+    <col min="9" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -597,7 +611,7 @@
       <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -1088,6 +1102,84 @@
       </c>
       <c r="I19" s="2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="4">
+        <v>45778</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0.52222222222222225</v>
+      </c>
+      <c r="E20" s="2">
+        <v>2063623</v>
+      </c>
+      <c r="F20" s="2">
+        <v>2063625</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H20" s="5">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4">
+        <v>45779</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0.57499999999999996</v>
+      </c>
+      <c r="E21" s="2">
+        <v>2063890</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="4">
+        <v>45779</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0.60347222222222219</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0.7104166666666667</v>
+      </c>
+      <c r="E22" s="2">
+        <v>2063966</v>
+      </c>
+      <c r="F22" s="2">
+        <v>2064230</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Now selecting glacier chain depending on summer, autumn temperature and winter precipitation. Added hindcast routing data. Adjusted plot files
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314436CA-9D01-464E-9EDF-277BD371C775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EAA67D3-9C67-D64D-AA5A-ED59DE0707E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="102980" yWindow="21860" windowWidth="30240" windowHeight="17360" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="900" yWindow="1080" windowWidth="32820" windowHeight="13940" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="58">
   <si>
     <t>Date</t>
   </si>
@@ -183,6 +183,33 @@
   </si>
   <si>
     <t>Rhb200</t>
+  </si>
+  <si>
+    <t>Glacier Comparison - test run, did not finish</t>
+  </si>
+  <si>
+    <t>Hd_2100, Hd_2150</t>
+  </si>
+  <si>
+    <t>Glacier Comparison - test run, did not finish, with sdbc</t>
+  </si>
+  <si>
+    <t>Glacier Comparison Low 2100</t>
+  </si>
+  <si>
+    <t>Ld_2100, Ln_2100</t>
+  </si>
+  <si>
+    <t>Glacier Comparison Md_2150</t>
+  </si>
+  <si>
+    <t>Md_2150</t>
+  </si>
+  <si>
+    <t>sund BC test future</t>
+  </si>
+  <si>
+    <t>Hd_2050, Hd_2100, Hd_2150, Ld_2100, Ln_2100, Md_2150</t>
   </si>
 </sst>
 </file>
@@ -577,7 +604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
@@ -1182,6 +1209,139 @@
         <v>22</v>
       </c>
     </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="4">
+        <v>45783</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0.69444444444444442</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.69513888888888886</v>
+      </c>
+      <c r="E23" s="2">
+        <v>2068515</v>
+      </c>
+      <c r="F23" s="2">
+        <v>2068516</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="4">
+        <v>45785</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0.37430555555555556</v>
+      </c>
+      <c r="E24" s="2">
+        <v>2071991</v>
+      </c>
+      <c r="F24" s="2">
+        <v>2071994</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="4">
+        <v>45785</v>
+      </c>
+      <c r="C25" s="3">
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="E25" s="2">
+        <v>2072063</v>
+      </c>
+      <c r="F25" s="2">
+        <v>2072065</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="4">
+        <v>45785</v>
+      </c>
+      <c r="C26" s="3">
+        <v>0.44305555555555554</v>
+      </c>
+      <c r="E26" s="2">
+        <v>2072074</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="4">
+        <v>45790</v>
+      </c>
+      <c r="C27" s="3">
+        <v>0.37708333333333333</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.38194444444444442</v>
+      </c>
+      <c r="E27" s="2">
+        <v>2075166</v>
+      </c>
+      <c r="F27" s="2">
+        <v>2075171</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
tested multiple variants match ch2018 chains to knmi chains; with and without trends. New boxplot functions for seasonal boxplots.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EAA67D3-9C67-D64D-AA5A-ED59DE0707E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DFEC89-346A-074A-82AD-8B3ECBC01FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="900" yWindow="1080" windowWidth="32820" windowHeight="13940" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="60">
   <si>
     <t>Date</t>
   </si>
@@ -210,6 +210,12 @@
   </si>
   <si>
     <t>Hd_2050, Hd_2100, Hd_2150, Ld_2100, Ln_2100, Md_2150</t>
+  </si>
+  <si>
+    <t>sund BC test future, did not finish</t>
+  </si>
+  <si>
+    <t>Future run glac V3</t>
   </si>
 </sst>
 </file>
@@ -604,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
@@ -1342,6 +1348,64 @@
         <v>12</v>
       </c>
     </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="4">
+        <v>45791</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0.44861111111111113</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.45347222222222222</v>
+      </c>
+      <c r="E28" s="2">
+        <v>2075520</v>
+      </c>
+      <c r="F28" s="2">
+        <v>2075525</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="4">
+        <v>45792</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="E29" s="2">
+        <v>2099863</v>
+      </c>
+      <c r="F29" s="2">
+        <v>2100021</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
overdue git update. plot info adjusted for presentation.
</commit_message>
<xml_diff>
--- a/hyperion/hyperion_jobs.xlsx
+++ b/hyperion/hyperion_jobs.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MT_case_sensitive/ETH_MT_Hydrological_Projections_Rhine_River/hyperion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DFEC89-346A-074A-82AD-8B3ECBC01FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2479E0CB-1E88-F54A-AE42-05C7C43B0476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1080" windowWidth="32820" windowHeight="13940" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
+    <workbookView xWindow="2560" yWindow="1060" windowWidth="29360" windowHeight="17920" xr2:uid="{35EEEF87-2CBF-EF4C-BD4A-04A9C12709A0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="imet_knmiens" sheetId="1" r:id="rId1"/>
+    <sheet name="ch_cumul_routing" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="102">
   <si>
     <t>Date</t>
   </si>
@@ -216,6 +217,132 @@
   </si>
   <si>
     <t>Future run glac V3</t>
+  </si>
+  <si>
+    <t>Future run glac V3 did not finish</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Thu200</t>
+  </si>
+  <si>
+    <t>WaS200</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>BEN200, Bod400, EmW200, HiR200, LaP200, Lim200, ThS200, Thu200</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>BiS200</t>
+  </si>
+  <si>
+    <t>Md_2100, Mn_2100</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>BiS200, Bod400, EmW200, LaP200, SeD200, TGl200, Rhb200</t>
+  </si>
+  <si>
+    <t>Hd_2050, Hn_2050</t>
+  </si>
+  <si>
+    <t>Md_2050, Mn_2050</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>SeD200, SSG200, TGl200, VoA200, VoR200, WaS200</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>ThS200, Thu200, BEN200, HiR200</t>
+  </si>
+  <si>
+    <t>Md_2050</t>
+  </si>
+  <si>
+    <t>VoA200, VoR200, WaS200</t>
+  </si>
+  <si>
+    <t>RhB200</t>
+  </si>
+  <si>
+    <t>Mn_2100</t>
+  </si>
+  <si>
+    <t>Gebiete_cumul</t>
+  </si>
+  <si>
+    <t>Gebiete_routing</t>
+  </si>
+  <si>
+    <t>SeD200, SSG200</t>
+  </si>
+  <si>
+    <t>Mn_2050</t>
+  </si>
+  <si>
+    <t>Hd_2150, Hn_2150</t>
+  </si>
+  <si>
+    <t>BEN200, BiS200, ThS200, Thu200</t>
+  </si>
+  <si>
+    <t>VoA200, WaS200</t>
+  </si>
+  <si>
+    <t>BEN200, HiR200, KEm200, Lim200, NeS200, SSG200, ThS200, Thu200, VoA200, VoR200</t>
+  </si>
+  <si>
+    <t>Md_2150, Mn_2150</t>
+  </si>
+  <si>
+    <t>SSG200</t>
+  </si>
+  <si>
+    <t>Hn_2150</t>
+  </si>
+  <si>
+    <t>BiS200, Bod400, EmW200, HiR200, KEm200, LaP200, Lim200</t>
+  </si>
+  <si>
+    <t>BEN200, BiS200, Bod400, EmW200, HiR200, KEm200, LaP200, Lim200</t>
+  </si>
+  <si>
+    <t>Md_2050, Md_2100, Mn2050</t>
+  </si>
+  <si>
+    <t>SSG200, ThS200</t>
+  </si>
+  <si>
+    <t>Mn_2150</t>
+  </si>
+  <si>
+    <t>Future run glac V3, nues cumulscripts</t>
+  </si>
+  <si>
+    <t>KeM200, Lim200</t>
+  </si>
+  <si>
+    <t>Hd_2050, Md_2150, Mn_2150</t>
+  </si>
+  <si>
+    <t>Future run glac V3, empty files</t>
+  </si>
+  <si>
+    <t>Future run glac V3, not full .RGS.gz</t>
   </si>
 </sst>
 </file>
@@ -268,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -276,6 +403,7 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -610,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460198F8-C33C-D741-968C-986857B440B6}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="2" customWidth="1"/>
@@ -1406,6 +1534,1332 @@
         <v>22</v>
       </c>
     </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="4">
+        <v>45793</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0.40486111111111112</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.45763888888888887</v>
+      </c>
+      <c r="E30" s="2">
+        <v>2103462</v>
+      </c>
+      <c r="F30" s="2">
+        <v>2103626</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="4">
+        <v>45794</v>
+      </c>
+      <c r="C31" s="3">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.56388888888888888</v>
+      </c>
+      <c r="E31" s="2">
+        <v>2104976</v>
+      </c>
+      <c r="F31" s="2">
+        <v>2105280</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="4">
+        <v>45794</v>
+      </c>
+      <c r="C32" s="3">
+        <v>0.68194444444444446</v>
+      </c>
+      <c r="E32" s="2">
+        <v>2105290</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="4">
+        <v>45794</v>
+      </c>
+      <c r="C33" s="3">
+        <v>0.68333333333333335</v>
+      </c>
+      <c r="E33" s="2">
+        <v>2105291</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="4">
+        <v>45794</v>
+      </c>
+      <c r="C34" s="3">
+        <v>0.68680555555555556</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0.68888888888888888</v>
+      </c>
+      <c r="E34" s="2">
+        <v>2105292</v>
+      </c>
+      <c r="F34" s="2">
+        <v>2105299</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="4">
+        <v>45794</v>
+      </c>
+      <c r="C35" s="3">
+        <v>0.69027777777777777</v>
+      </c>
+      <c r="E35" s="2">
+        <v>2105300</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="4">
+        <v>45795</v>
+      </c>
+      <c r="C36" s="3">
+        <v>0.8979166666666667</v>
+      </c>
+      <c r="D36" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="E36" s="2">
+        <v>2146511</v>
+      </c>
+      <c r="F36" s="2">
+        <v>2146822</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="4">
+        <v>45796</v>
+      </c>
+      <c r="C37" s="3">
+        <v>0.35694444444444445</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0.35972222222222222</v>
+      </c>
+      <c r="E37" s="2">
+        <v>2146823</v>
+      </c>
+      <c r="F37" s="2">
+        <v>2146829</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38" s="4">
+        <v>45796</v>
+      </c>
+      <c r="C38" s="3">
+        <v>0.3659722222222222</v>
+      </c>
+      <c r="D38" s="3">
+        <v>0.47152777777777777</v>
+      </c>
+      <c r="E38" s="2">
+        <v>2146840</v>
+      </c>
+      <c r="F38" s="2">
+        <v>2147144</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" s="4">
+        <v>45796</v>
+      </c>
+      <c r="C39" s="3">
+        <v>0.84375</v>
+      </c>
+      <c r="D39" s="3">
+        <v>0.94930555555555551</v>
+      </c>
+      <c r="E39" s="2">
+        <v>2147267</v>
+      </c>
+      <c r="F39" s="2">
+        <v>2147574</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C40" s="3">
+        <v>0.39513888888888887</v>
+      </c>
+      <c r="E40" s="2">
+        <v>2147586</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B41" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C41" s="3">
+        <v>0.42083333333333334</v>
+      </c>
+      <c r="D41" s="3">
+        <v>0.42222222222222222</v>
+      </c>
+      <c r="E41" s="2">
+        <v>2147587</v>
+      </c>
+      <c r="F41" s="2">
+        <v>2147592</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B42" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C42" s="3">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="D42" s="3">
+        <v>0.42499999999999999</v>
+      </c>
+      <c r="E42" s="2">
+        <v>2147593</v>
+      </c>
+      <c r="F42" s="2">
+        <v>2147596</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C43" s="3">
+        <v>0.42638888888888887</v>
+      </c>
+      <c r="E43" s="2">
+        <v>2147597</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C44" s="3">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="E44" s="2">
+        <v>2147598</v>
+      </c>
+      <c r="F44" s="2">
+        <v>2147600</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B45" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C45" s="3">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="E45" s="2">
+        <v>2147601</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0.43472222222222223</v>
+      </c>
+      <c r="E46" s="2">
+        <v>2147602</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C47" s="3">
+        <v>0.55138888888888893</v>
+      </c>
+      <c r="E47" s="2">
+        <v>2147625</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C48" s="3">
+        <v>0.56319444444444444</v>
+      </c>
+      <c r="D48" s="3">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="E48" s="2">
+        <v>2147626</v>
+      </c>
+      <c r="F48" s="2">
+        <v>2147643</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B49" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C49" s="3">
+        <v>0.66874999999999996</v>
+      </c>
+      <c r="D49" s="3">
+        <v>0.6694444444444444</v>
+      </c>
+      <c r="E49" s="2">
+        <v>2147669</v>
+      </c>
+      <c r="F49" s="2">
+        <v>2147670</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C50" s="3">
+        <v>0.6743055555555556</v>
+      </c>
+      <c r="E50" s="2">
+        <v>2147671</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C51" s="3">
+        <v>0.73472222222222228</v>
+      </c>
+      <c r="E51" s="2">
+        <v>2147681</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="4">
+        <v>45797</v>
+      </c>
+      <c r="C52" s="3">
+        <v>0.7368055555555556</v>
+      </c>
+      <c r="D52" s="3">
+        <v>0.84166666666666667</v>
+      </c>
+      <c r="E52" s="2">
+        <v>2147682</v>
+      </c>
+      <c r="F52" s="2">
+        <v>2147986</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="4">
+        <v>45798</v>
+      </c>
+      <c r="C53" s="3">
+        <v>0.37361111111111112</v>
+      </c>
+      <c r="D53" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="E53" s="2">
+        <v>2147987</v>
+      </c>
+      <c r="F53" s="2">
+        <v>2147992</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B54" s="4">
+        <v>45798</v>
+      </c>
+      <c r="C54" s="3">
+        <v>0.37638888888888888</v>
+      </c>
+      <c r="D54" s="3">
+        <v>0.37708333333333333</v>
+      </c>
+      <c r="E54" s="2">
+        <v>2147993</v>
+      </c>
+      <c r="F54" s="2">
+        <v>2147996</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55" s="4">
+        <v>45798</v>
+      </c>
+      <c r="C55" s="3">
+        <v>0.37916666666666665</v>
+      </c>
+      <c r="E55" s="2">
+        <v>2147998</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B56" s="4">
+        <v>45798</v>
+      </c>
+      <c r="C56" s="3">
+        <v>0.74097222222222225</v>
+      </c>
+      <c r="D56" s="3">
+        <v>0.74097222222222225</v>
+      </c>
+      <c r="E56" s="2">
+        <v>2148012</v>
+      </c>
+      <c r="F56" s="2">
+        <v>2148013</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H56" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B57" s="4">
+        <v>45798</v>
+      </c>
+      <c r="C57" s="3">
+        <v>0.74583333333333335</v>
+      </c>
+      <c r="D57" s="3">
+        <v>0.74930555555555556</v>
+      </c>
+      <c r="E57" s="2">
+        <v>2148014</v>
+      </c>
+      <c r="F57" s="2">
+        <v>2148023</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H57" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" s="4">
+        <v>45798</v>
+      </c>
+      <c r="C58" s="3">
+        <v>0.75069444444444444</v>
+      </c>
+      <c r="D58" s="3">
+        <v>0.85624999999999996</v>
+      </c>
+      <c r="E58" s="2">
+        <v>2148024</v>
+      </c>
+      <c r="F58" s="2">
+        <v>2148330</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H58" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59" s="4">
+        <v>45799</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0.34583333333333333</v>
+      </c>
+      <c r="E59" s="2">
+        <v>2148331</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H59" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B60" s="4">
+        <v>45799</v>
+      </c>
+      <c r="C60" s="3">
+        <v>0.35347222222222224</v>
+      </c>
+      <c r="D60" s="3">
+        <v>0.35555555555555557</v>
+      </c>
+      <c r="E60" s="2">
+        <v>2148332</v>
+      </c>
+      <c r="F60" s="2">
+        <v>2148338</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H60" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B61" s="4">
+        <v>45799</v>
+      </c>
+      <c r="C61" s="3">
+        <v>0.35694444444444445</v>
+      </c>
+      <c r="D61" s="3">
+        <v>0.35902777777777778</v>
+      </c>
+      <c r="E61" s="2">
+        <v>2148339</v>
+      </c>
+      <c r="F61" s="2">
+        <v>2148346</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H61" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="4">
+        <v>45799</v>
+      </c>
+      <c r="C62" s="3">
+        <v>0.57777777777777772</v>
+      </c>
+      <c r="E62" s="2">
+        <v>2148881</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H62" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63" s="4">
+        <v>45800</v>
+      </c>
+      <c r="C63" s="3">
+        <v>0.39374999999999999</v>
+      </c>
+      <c r="D63" s="3">
+        <v>0.39444444444444443</v>
+      </c>
+      <c r="E63" s="2">
+        <v>2149474</v>
+      </c>
+      <c r="F63" s="2">
+        <v>2149475</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H63" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64" s="4">
+        <v>45800</v>
+      </c>
+      <c r="C64" s="3">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E64" s="2">
+        <v>2149476</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H64" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B65" s="4">
+        <v>45800</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="E65" s="2">
+        <v>2149477</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H65" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B66" s="4">
+        <v>45800</v>
+      </c>
+      <c r="C66" s="3">
+        <v>0.42152777777777778</v>
+      </c>
+      <c r="E66" s="2">
+        <v>2149479</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H66" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B67" s="4">
+        <v>45803</v>
+      </c>
+      <c r="C67" s="3">
+        <v>0.86944444444444446</v>
+      </c>
+      <c r="D67" s="3">
+        <v>0.86944444444444446</v>
+      </c>
+      <c r="E67" s="2">
+        <v>2151808</v>
+      </c>
+      <c r="F67" s="2">
+        <v>2151809</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H67" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B68" s="4">
+        <v>45808</v>
+      </c>
+      <c r="C68" s="3">
+        <v>0.67986111111111114</v>
+      </c>
+      <c r="E68" s="2">
+        <v>2154468</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H68" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D204BF92-0F32-3440-9BB6-EF17DF445493}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="7">
+        <v>45797</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="7">
+        <v>45797</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="7">
+        <v>45797</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="7">
+        <v>45797</v>
+      </c>
+      <c r="C5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="7">
+        <v>45798</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="7">
+        <v>45799</v>
+      </c>
+      <c r="C7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="7">
+        <v>45800</v>
+      </c>
+      <c r="C8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="7">
+        <v>45800</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="7">
+        <v>45800</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="7">
+        <v>45800</v>
+      </c>
+      <c r="C11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="7">
+        <v>45804</v>
+      </c>
+      <c r="C12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="7">
+        <v>45806</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="7">
+        <v>45808</v>
+      </c>
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="F14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B15" s="7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>